<commit_message>
Data dictionary: fill and correct value definitions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/aaron_skinner2_ubc_ca/Documents/Academia/PhD/Analysis/Ssp-bird-data-wrangling/DataS1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94C0018A-6AE8-1D4C-B457-BDCFEEAC2453}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E151FD8F-A58E-CA40-BF32-592B29B239E8}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bird_pcs_all" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="219">
   <si>
     <t>Field_name</t>
   </si>
@@ -325,13 +325,6 @@
     <t>Name of the data collector</t>
   </si>
   <si>
-    <t>CIPAV: Centro para la Investigación en Sistemas Sostenibles de Producción Agropecuaria
-GAICA: Asociación GAICA 
-UBC GAICA: The University of British Columbia and Asociación GAICA
-UniLlanos: Universidad de los Llanos
-UBC: The University of British Columbia</t>
-  </si>
-  <si>
     <t>Uniq_db</t>
   </si>
   <si>
@@ -355,9 +348,6 @@
     <t>Years grouped together by major sampling effort</t>
   </si>
   <si>
-    <t>Five major periods of bird data collection (2013-2014, 2016-2017, 2019, 2022, 2024)</t>
-  </si>
-  <si>
     <t>Year</t>
   </si>
   <si>
@@ -411,12 +401,6 @@
     <t>Weather</t>
   </si>
   <si>
-    <t>Despejado: Clear
-Nublado: Cloudy
-Brisa: Breeze
-Llovizna: Drizzling</t>
-  </si>
-  <si>
     <t>Cows_50m</t>
   </si>
   <si>
@@ -430,10 +414,6 @@
   </si>
   <si>
     <t>Season</t>
-  </si>
-  <si>
-    <t>Early = within 80 days of the first survey in that Ano_grp
-Late = 80+ days after</t>
   </si>
   <si>
     <t>Sampling_day</t>
@@ -512,200 +492,224 @@
     <t>Habitat subtype</t>
   </si>
   <si>
+    <t>Id_group_no_dc</t>
+  </si>
+  <si>
+    <t>A cluster of point counts on a single farm, irrespective of the data collector</t>
+  </si>
+  <si>
+    <t>Farm_name</t>
+  </si>
+  <si>
+    <t>Name of the farm where the point count was located</t>
+  </si>
+  <si>
+    <t>Distance_farm</t>
+  </si>
+  <si>
+    <t>Generation length</t>
+  </si>
+  <si>
+    <t>Bird et al. 2020</t>
+  </si>
+  <si>
+    <t>IUCN Red List category</t>
+  </si>
+  <si>
+    <t>HBW/BirdLife checklist</t>
+  </si>
+  <si>
+    <t>Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
+  </si>
+  <si>
+    <t>Dense (forest interior, thickets); Semi_open (open shrubland, parkland, thorn forest); Open (desert, grassland, open water, rocky habitat, cities, forest canopy)</t>
+  </si>
+  <si>
+    <t>Herbivore; Carnivore; Scavenger; Omnivore</t>
+  </si>
+  <si>
+    <t>Frugivore; Granivore; Nectarivore; Herbivore; Herbivore aquatic; Invertivore; Vertivore; Aquatic predator; Scavenger; Omnivore</t>
+  </si>
+  <si>
+    <t>Aerial (mostly in flight); Terrestrial (on the ground); Insessorial (perching above ground); Aquatic (on water); Generalist</t>
+  </si>
+  <si>
+    <t>Tarsus length (mm)</t>
+  </si>
+  <si>
+    <t>Unflattened wing length (mm)</t>
+  </si>
+  <si>
+    <t>100 x Kipp's distance / wing length</t>
+  </si>
+  <si>
+    <t>Tail length (mm)</t>
+  </si>
+  <si>
+    <t>Species mean mass (g) across sexes</t>
+  </si>
+  <si>
+    <t>Migratory status AVONET</t>
+  </si>
+  <si>
+    <t>Migratory status BIRDBASE</t>
+  </si>
+  <si>
+    <t>Primary diet category</t>
+  </si>
+  <si>
+    <t>Number of major food groups used</t>
+  </si>
+  <si>
+    <t>Number of major habitat types used</t>
+  </si>
+  <si>
+    <t>Ecological specialization index</t>
+  </si>
+  <si>
+    <t>Minimum clutch size</t>
+  </si>
+  <si>
+    <t>Maximum clutch size</t>
+  </si>
+  <si>
+    <t>Mean of clutch_min and clutch_max</t>
+  </si>
+  <si>
+    <t>Elevational range width</t>
+  </si>
+  <si>
+    <t>Species name according to BirdLife International</t>
+  </si>
+  <si>
+    <t>From HBW-BirdLife checklist v5, Dec 2020</t>
+  </si>
+  <si>
+    <t>Number of individuals measured for the species</t>
+  </si>
+  <si>
+    <t>Length from base of the skull to tip of beak (mm)</t>
+  </si>
+  <si>
+    <t>Length from the anterior edge of the nostrils to the tip of beak (mm)</t>
+  </si>
+  <si>
+    <t>Width at the anterior edge of the nostrils (mm)</t>
+  </si>
+  <si>
+    <t>Depth at the anterior edge of the nostrils (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predominant habitat type occupied </t>
+  </si>
+  <si>
+    <t>Openness of predominant habitat</t>
+  </si>
+  <si>
+    <t>Broad trophic category</t>
+  </si>
+  <si>
+    <t>Predominant resource used</t>
+  </si>
+  <si>
+    <t>Predominant locomotion / foraging substrate</t>
+  </si>
+  <si>
+    <t>Minimum latitude of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Maximum latitude of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Area of breeding and resident range (km^2)</t>
+  </si>
+  <si>
+    <t>Distance from secondary1 to the longest primary (mm)</t>
+  </si>
+  <si>
+    <t>Length from carpal joint to tip of secondary1 (mm)</t>
+  </si>
+  <si>
+    <t>Latitude of centroid of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Longitude of centroid of breeding and resident range (decimal degrees)</t>
+  </si>
+  <si>
+    <t>Species Latin name according to Ayerbe's 2018 field guide</t>
+  </si>
+  <si>
+    <t>Annual precipitation (millimeters)</t>
+  </si>
+  <si>
+    <t>Distance (m) from the point count to the nearest farm boundary</t>
+  </si>
+  <si>
+    <t>Pc_duration</t>
+  </si>
+  <si>
+    <t>Number of distinct 'Year_grp's sampled</t>
+  </si>
+  <si>
+    <t>Point count repetition number within Year_grp</t>
+  </si>
+  <si>
+    <t>Weather categories</t>
+  </si>
+  <si>
+    <t>Whether the survey fell within an 80-day sampling window relative to the first survey of that Year_grp</t>
+  </si>
+  <si>
+    <t>Point count repetition number within a season</t>
+  </si>
+  <si>
+    <t>Day number within a closed sampling period, per institution and Year_grp</t>
+  </si>
+  <si>
+    <t>N_visits</t>
+  </si>
+  <si>
+    <t>Total number of surveys at a point count location</t>
+  </si>
+  <si>
+    <t>Percent canopy cover within a 1 km buffer, see Potapov et al. (2026)</t>
+  </si>
+  <si>
+    <t>Max canopy height (in meters) within the point count buffer, see Potapov et al. (2026)</t>
+  </si>
+  <si>
+    <t>See Table 3 in the main text</t>
+  </si>
+  <si>
+    <t>Despejado: Clear
+Nublado: Cloudy
+Brisa: Breeze
+Lluvia: Rain
+Llovizna: Drizzling</t>
+  </si>
+  <si>
     <t>Maduro = Mature forest
 Ripario = Riparian forest
 Secundario = Secondary forest
 Arboles dispersos = Dispersed trees
 Cerca viva = Live fence
-Banco de forraje = Forrage bank
-Setos = Live fence of (foraging) bushes
-Intensivo = Intensive  silvopastoral system</t>
-  </si>
-  <si>
-    <t>Id_group_no_dc</t>
-  </si>
-  <si>
-    <t>A cluster of point counts on a single farm, irrespective of the data collector</t>
-  </si>
-  <si>
-    <t>Farm_name</t>
-  </si>
-  <si>
-    <t>Name of the farm where the point count was located</t>
-  </si>
-  <si>
-    <t>Distance_farm</t>
-  </si>
-  <si>
-    <t>Generation length</t>
-  </si>
-  <si>
-    <t>Bird et al. 2020</t>
-  </si>
-  <si>
-    <t>IUCN Red List category</t>
-  </si>
-  <si>
-    <t>HBW/BirdLife checklist</t>
-  </si>
-  <si>
-    <t>Desert; Rock; Grassland; Shrubland; Woodland; Forest; Human Modified; Wetland; Riverine; Coastal; Marine</t>
-  </si>
-  <si>
-    <t>Dense (forest interior, thickets); Semi_open (open shrubland, parkland, thorn forest); Open (desert, grassland, open water, rocky habitat, cities, forest canopy)</t>
-  </si>
-  <si>
-    <t>Herbivore; Carnivore; Scavenger; Omnivore</t>
-  </si>
-  <si>
-    <t>Frugivore; Granivore; Nectarivore; Herbivore; Herbivore aquatic; Invertivore; Vertivore; Aquatic predator; Scavenger; Omnivore</t>
-  </si>
-  <si>
-    <t>Aerial (mostly in flight); Terrestrial (on the ground); Insessorial (perching above ground); Aquatic (on water); Generalist</t>
-  </si>
-  <si>
-    <t>Tarsus length (mm)</t>
-  </si>
-  <si>
-    <t>Unflattened wing length (mm)</t>
-  </si>
-  <si>
-    <t>100 x Kipp's distance / wing length</t>
-  </si>
-  <si>
-    <t>Tail length (mm)</t>
-  </si>
-  <si>
-    <t>Species mean mass (g) across sexes</t>
-  </si>
-  <si>
-    <t>Migratory status AVONET</t>
-  </si>
-  <si>
-    <t>Migratory status BIRDBASE</t>
-  </si>
-  <si>
-    <t>Primary diet category</t>
-  </si>
-  <si>
-    <t>Number of major food groups used</t>
-  </si>
-  <si>
-    <t>Number of major habitat types used</t>
-  </si>
-  <si>
-    <t>Ecological specialization index</t>
-  </si>
-  <si>
-    <t>Minimum clutch size</t>
-  </si>
-  <si>
-    <t>Maximum clutch size</t>
-  </si>
-  <si>
-    <t>Mean of clutch_min and clutch_max</t>
-  </si>
-  <si>
-    <t>Elevational range width</t>
-  </si>
-  <si>
-    <t>Species name according to BirdLife International</t>
-  </si>
-  <si>
-    <t>From HBW-BirdLife checklist v5, Dec 2020</t>
-  </si>
-  <si>
-    <t>Number of individuals measured for the species</t>
-  </si>
-  <si>
-    <t>Length from base of the skull to tip of beak (mm)</t>
-  </si>
-  <si>
-    <t>Length from the anterior edge of the nostrils to the tip of beak (mm)</t>
-  </si>
-  <si>
-    <t>Width at the anterior edge of the nostrils (mm)</t>
-  </si>
-  <si>
-    <t>Depth at the anterior edge of the nostrils (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predominant habitat type occupied </t>
-  </si>
-  <si>
-    <t>Openness of predominant habitat</t>
-  </si>
-  <si>
-    <t>Broad trophic category</t>
-  </si>
-  <si>
-    <t>Predominant resource used</t>
-  </si>
-  <si>
-    <t>Predominant locomotion / foraging substrate</t>
-  </si>
-  <si>
-    <t>Minimum latitude of breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Maximum latitude of breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Area of breeding and resident range (km^2)</t>
-  </si>
-  <si>
-    <t>Distance from secondary1 to the longest primary (mm)</t>
-  </si>
-  <si>
-    <t>Length from carpal joint to tip of secondary1 (mm)</t>
-  </si>
-  <si>
-    <t>Latitude of centroid of breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Longitude of centroid of breeding and resident range (decimal degrees)</t>
-  </si>
-  <si>
-    <t>Species Latin name according to Ayerbe's 2018 field guide</t>
-  </si>
-  <si>
-    <t>Annual precipitation (millimeters)</t>
-  </si>
-  <si>
-    <t>Distance (m) from the point count to the nearest farm boundary</t>
-  </si>
-  <si>
-    <t>Pc_duration</t>
-  </si>
-  <si>
-    <t>Number of distinct 'Year_grp's sampled</t>
-  </si>
-  <si>
-    <t>Point count repetition number within Year_grp</t>
-  </si>
-  <si>
-    <t>Weather categories</t>
-  </si>
-  <si>
-    <t>Whether the survey fell within an 80-day sampling window relative to the first survey of that Year_grp</t>
-  </si>
-  <si>
-    <t>Point count repetition number within a season</t>
-  </si>
-  <si>
-    <t>Day number within a closed sampling period, per institution and Year_grp</t>
-  </si>
-  <si>
-    <t>N_visits</t>
-  </si>
-  <si>
-    <t>Total number of surveys at a point count location</t>
-  </si>
-  <si>
-    <t>Percent canopy cover within a 1 km buffer, see Potapov et al. (2026)</t>
-  </si>
-  <si>
-    <t>Max canopy height (in meters) within the point count buffer, see Potapov et al. (2026)</t>
+Banco de forraje = Forage bank
+Setos = Shrub live fence (i.e., hedgerow)
+Intensivo = Intensive silvopastoral system</t>
+  </si>
+  <si>
+    <t>Six major periods of bird data collection (2013-2014, 2016-2017, 2019, 2022, 2024, 2025-2026)</t>
+  </si>
+  <si>
+    <t>Early = within 80 days of the first survey in that Year_grp
+Late = 80+ days after</t>
+  </si>
+  <si>
+    <t>Cipav: Centro para la Investigación en Sistemas Sostenibles de Producción Agropecuaria
+Gaica: Asociación GAICA 
+Ubc gaica: The University of British Columbia and Asociación GAICA
+Unillanos: Universidad de los Llanos
+Ubc: The University of British Columbia</t>
   </si>
 </sst>
 </file>
@@ -741,8 +745,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1096,7 +1103,7 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1150,6 +1157,7 @@
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="129.1640625" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -1182,34 +1190,34 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="144" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>96</v>
       </c>
       <c r="B4" t="s">
         <v>97</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>99</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="C5" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" t="s">
         <v>102</v>
-      </c>
-      <c r="B6" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -1222,45 +1230,45 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
         <v>104</v>
       </c>
-      <c r="B8" t="s">
-        <v>105</v>
-      </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -1273,129 +1281,129 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B15" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B17" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
-        <v>211</v>
-      </c>
-      <c r="C18" t="s">
-        <v>130</v>
+        <v>206</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" t="s">
         <v>117</v>
       </c>
-      <c r="B19" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="C20" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B20" t="s">
-        <v>119</v>
-      </c>
-      <c r="C20" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>121</v>
       </c>
-      <c r="B21" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>123</v>
-      </c>
       <c r="B22" t="s">
-        <v>210</v>
-      </c>
-      <c r="C22" t="s">
-        <v>124</v>
+        <v>205</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B24" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B25" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C25" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B26" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C26" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B27" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C27" t="s">
         <v>76</v>
@@ -1413,6 +1421,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="51.1640625" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -1436,120 +1445,123 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>135</v>
+      </c>
+      <c r="C4" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B7" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B8" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B11" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B13" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B14" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="80" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>151</v>
-      </c>
-      <c r="C15" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="160" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C16" t="s">
-        <v>155</v>
+        <v>150</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -1599,13 +1611,13 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C3" t="s">
         <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1613,7 +1625,7 @@
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
@@ -1624,7 +1636,7 @@
         <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -1635,7 +1647,7 @@
         <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
@@ -1646,7 +1658,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -1657,7 +1669,7 @@
         <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
@@ -1668,7 +1680,7 @@
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
@@ -1679,7 +1691,7 @@
         <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
         <v>36</v>
@@ -1690,7 +1702,7 @@
         <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1701,7 +1713,7 @@
         <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -1712,7 +1724,7 @@
         <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
@@ -1723,7 +1735,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C14" t="s">
         <v>36</v>
@@ -1734,7 +1746,7 @@
         <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C15" t="s">
         <v>36</v>
@@ -1745,13 +1757,13 @@
         <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C16" t="s">
         <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -1759,13 +1771,13 @@
         <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C17" t="s">
         <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1773,13 +1785,13 @@
         <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C18" t="s">
         <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -1787,13 +1799,13 @@
         <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C19" t="s">
         <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -1801,13 +1813,13 @@
         <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C20" t="s">
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -1815,7 +1827,7 @@
         <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
@@ -1826,7 +1838,7 @@
         <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -1837,7 +1849,7 @@
         <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C23" t="s">
         <v>36</v>
@@ -1848,7 +1860,7 @@
         <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C24" t="s">
         <v>36</v>
@@ -1859,7 +1871,7 @@
         <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C25" t="s">
         <v>36</v>
@@ -1881,7 +1893,7 @@
         <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C27" t="s">
         <v>36</v>
@@ -1895,7 +1907,7 @@
         <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C28" t="s">
         <v>63</v>
@@ -1909,7 +1921,7 @@
         <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
         <v>63</v>
@@ -1920,7 +1932,7 @@
         <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C30" t="s">
         <v>63</v>
@@ -1931,7 +1943,7 @@
         <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="C31" t="s">
         <v>63</v>
@@ -1942,7 +1954,7 @@
         <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C32" t="s">
         <v>63</v>
@@ -1956,7 +1968,7 @@
         <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C33" t="s">
         <v>63</v>
@@ -1967,7 +1979,7 @@
         <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C34" t="s">
         <v>63</v>
@@ -1978,7 +1990,7 @@
         <v>72</v>
       </c>
       <c r="B35" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C35" t="s">
         <v>63</v>
@@ -1989,10 +2001,10 @@
         <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C36" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D36" t="s">
         <v>74</v>
@@ -2003,7 +2015,7 @@
         <v>75</v>
       </c>
       <c r="B37" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C37" t="s">
         <v>33</v>
@@ -2017,10 +2029,10 @@
         <v>77</v>
       </c>
       <c r="B38" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C38" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explain the deposit's blank cells as NA, not recorded, or missing
- The metadata tables split blanks three ways using a rule per column, and report blank counts for every column type.
- Integer type comes from a named list of count columns, so rounded measurements stay numeric.
- Dictionary edits: blank-cell definitions, "In field", Spp_obs Yes/No.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/aaron_skinner2_ubc_ca/Documents/Academia/PhD/Analysis/Ssp-bird-data-wrangling/DataS1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="96" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E151FD8F-A58E-CA40-BF32-592B29B239E8}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36ADA9C1-E8BC-CE41-8F1B-134B935CD0C9}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25120" windowHeight="14840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1660" yWindow="660" windowWidth="25120" windowHeight="13180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bird_pcs_all" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="229">
   <si>
     <t>Field_name</t>
   </si>
@@ -248,9 +248,6 @@
     <t>Gen_length</t>
   </si>
   <si>
-    <t>Years</t>
-  </si>
-  <si>
     <t>Elev_range</t>
   </si>
   <si>
@@ -293,30 +290,16 @@
     <t>Distance_bird</t>
   </si>
   <si>
-    <t>The distance to the bird from the observer</t>
-  </si>
-  <si>
     <t>Obs_type</t>
   </si>
   <si>
     <t>How bird was identified</t>
   </si>
   <si>
-    <t>Auditivo: By ear
-Sobrevuelo: Bird flew over and did not use the habitat
-Tamborileo: Drumming
-Visual: By sight
-Visual/auditivo: By sight and by ear</t>
-  </si>
-  <si>
     <t>Recording</t>
   </si>
   <si>
     <t>Whether species was identified in a recording</t>
-  </si>
-  <si>
-    <t>Cf: A bird that was identified in the field and was confirmed in the recording 
-Y: A bird that was only identified in the recording</t>
   </si>
   <si>
     <t>Institution_name</t>
@@ -385,11 +368,6 @@
   </si>
   <si>
     <t>Whether any species were observed at the point count</t>
-  </si>
-  <si>
-    <t>0 = No species observed during point count
-1 = Species were observed during point count
-NOTE: Based on the Bird_pcs_all file, not the Bird_pcs_analysis file</t>
   </si>
   <si>
     <t>Noise</t>
@@ -507,9 +485,6 @@
     <t>Distance_farm</t>
   </si>
   <si>
-    <t>Generation length</t>
-  </si>
-  <si>
     <t>Bird et al. 2020</t>
   </si>
   <si>
@@ -576,9 +551,6 @@
     <t>Mean of clutch_min and clutch_max</t>
   </si>
   <si>
-    <t>Elevational range width</t>
-  </si>
-  <si>
     <t>Species name according to BirdLife International</t>
   </si>
   <si>
@@ -679,13 +651,74 @@
   </si>
   <si>
     <t>See Table 3 in the main text</t>
+  </si>
+  <si>
+    <t>Six major periods of bird data collection (2013-2014, 2016-2017, 2019, 2022, 2024, 2025-2026)</t>
+  </si>
+  <si>
+    <t>Early = within 80 days of the first survey in that Year_grp
+Late = 80+ days after</t>
+  </si>
+  <si>
+    <t>Cipav: Centro para la Investigación en Sistemas Sostenibles de Producción Agropecuaria
+Gaica: Asociación GAICA 
+Ubc gaica: The University of British Columbia and Asociación GAICA
+Unillanos: Universidad de los Llanos
+Ubc: The University of British Columbia</t>
+  </si>
+  <si>
+    <t>Unique point count ID</t>
+  </si>
+  <si>
+    <t>The distance from the observer to the bird</t>
+  </si>
+  <si>
+    <t>No = No species observed during point count
+Yes = Species were observed during point count
+NOTE: Based on the Bird_pcs_all file, not the Bird_pcs_analysis file</t>
+  </si>
+  <si>
+    <t>NA = no farm ID (Otún Quimbaya reserve)</t>
+  </si>
+  <si>
+    <t>Auditivo: By ear
+Sobrevuelo: Bird flew over and did not use the habitat
+Tamborileo: Drumming
+Visual: By sight
+Visual/auditivo: By sight and by ear
+blank: CIPAV did not record, otherwise missing</t>
+  </si>
+  <si>
+    <t>blank: generally not recorded, otherwise missing if associated with UBC</t>
   </si>
   <si>
     <t>Despejado: Clear
 Nublado: Cloudy
 Brisa: Breeze
 Lluvia: Rain
-Llovizna: Drizzling</t>
+Llovizna: Drizzling
+blank: not recorded by CIPAV or GAICA mbd; otherwise missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cf: A bird that was identified in the field and was confirmed in the recording 
+Y: A bird that was only identified in the recording
+In field: Identified in the field only
+blank: Not recorded - recordings were made only by UBC-GAICA in the Eje cafetero, 2024. </t>
+  </si>
+  <si>
+    <t>blank: NA for detections identified only from the recording (no field count), otherwise missing.</t>
+  </si>
+  <si>
+    <t>NA = no associated farm (Otún Quimbaya reserve)</t>
+  </si>
+  <si>
+    <t>blank: missing</t>
+  </si>
+  <si>
+    <t>blank: one CIPAV point with a single observation</t>
+  </si>
+  <si>
+    <t>NA: not in SACC 2018</t>
   </si>
   <si>
     <t>Maduro = Mature forest
@@ -695,21 +728,25 @@
 Cerca viva = Live fence
 Banco de forraje = Forage bank
 Setos = Shrub live fence (i.e., hedgerow)
-Intensivo = Intensive silvopastoral system</t>
-  </si>
-  <si>
-    <t>Six major periods of bird data collection (2013-2014, 2016-2017, 2019, 2022, 2024, 2025-2026)</t>
-  </si>
-  <si>
-    <t>Early = within 80 days of the first survey in that Year_grp
-Late = 80+ days after</t>
-  </si>
-  <si>
-    <t>Cipav: Centro para la Investigación en Sistemas Sostenibles de Producción Agropecuaria
-Gaica: Asociación GAICA 
-Ubc gaica: The University of British Columbia and Asociación GAICA
-Unillanos: Universidad de los Llanos
-Ubc: The University of British Columbia</t>
+Intensivo = Intensive silvopastoral system
+NA = not applicable (crops, mosaic, intensive pasture)</t>
+  </si>
+  <si>
+    <t>A continuous distance (m) or a distance class (&lt;25, &lt;50, &gt;50; 0-15, 15-30, 30-50). Flyovers have an estimated distance or class in most datasets, but are blank for GAICA mbd 2013 and UBC-GAICA. 
+NA: flyover (no distance estimated)
+blank: missing</t>
+  </si>
+  <si>
+    <t>missing: not available in bird base</t>
+  </si>
+  <si>
+    <t>Elevational range width (meters)</t>
+  </si>
+  <si>
+    <t>missing: Pheucticus ludovicianus, no elevational range in any source</t>
+  </si>
+  <si>
+    <t>Generation length (Years)</t>
   </si>
 </sst>
 </file>
@@ -1046,13 +1083,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="59.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1063,85 +1101,92 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C2" t="s">
         <v>79</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>81</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>83</v>
       </c>
-      <c r="B4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>84</v>
       </c>
-      <c r="B5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" t="s">
         <v>86</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" ht="96" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>88</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="C9" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>90</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>91</v>
       </c>
-      <c r="C9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C10" t="s">
-        <v>95</v>
+      <c r="C10" s="1" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -1156,7 +1201,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="129.1640625" customWidth="1"/>
+    <col min="2" max="2" width="61.83203125" customWidth="1"/>
     <col min="3" max="3" width="28.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1173,240 +1218,252 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" t="s">
         <v>78</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>79</v>
-      </c>
-      <c r="C2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" t="s">
         <v>81</v>
-      </c>
-      <c r="B3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="144" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="96" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C8" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" t="s">
         <v>84</v>
-      </c>
-      <c r="B13" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>106</v>
+      </c>
+      <c r="C14" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B17" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B18" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="96" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>118</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+      <c r="C21" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="112" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B22" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B23" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="C23" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B24" t="s">
-        <v>125</v>
+        <v>120</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B25" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C25" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B26" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C26" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B27" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1437,109 +1494,115 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" t="s">
         <v>81</v>
-      </c>
-      <c r="B2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>128</v>
+      </c>
+      <c r="C3" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C4" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B8" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B9" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B10" t="s">
-        <v>201</v>
+        <v>194</v>
+      </c>
+      <c r="C10" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B11" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B12" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B14" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="80" x14ac:dyDescent="0.2">
@@ -1547,21 +1610,21 @@
         <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="160" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="192" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -1611,13 +1674,13 @@
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
         <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1625,7 +1688,7 @@
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
@@ -1636,7 +1699,7 @@
         <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
@@ -1647,7 +1710,7 @@
         <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
@@ -1658,7 +1721,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -1669,7 +1732,7 @@
         <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
@@ -1680,7 +1743,7 @@
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
@@ -1691,7 +1754,7 @@
         <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C10" t="s">
         <v>36</v>
@@ -1702,7 +1765,7 @@
         <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1713,7 +1776,7 @@
         <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -1724,7 +1787,7 @@
         <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
@@ -1735,7 +1798,7 @@
         <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C14" t="s">
         <v>36</v>
@@ -1746,7 +1809,7 @@
         <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C15" t="s">
         <v>36</v>
@@ -1757,13 +1820,13 @@
         <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C16" t="s">
         <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -1771,13 +1834,13 @@
         <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="C17" t="s">
         <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1785,13 +1848,13 @@
         <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C18" t="s">
         <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -1799,13 +1862,13 @@
         <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C19" t="s">
         <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -1813,13 +1876,13 @@
         <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C20" t="s">
         <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -1827,7 +1890,7 @@
         <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
@@ -1838,7 +1901,7 @@
         <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -1849,7 +1912,7 @@
         <v>55</v>
       </c>
       <c r="B23" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="C23" t="s">
         <v>36</v>
@@ -1860,7 +1923,7 @@
         <v>56</v>
       </c>
       <c r="B24" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C24" t="s">
         <v>36</v>
@@ -1871,7 +1934,7 @@
         <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="C25" t="s">
         <v>36</v>
@@ -1893,7 +1956,7 @@
         <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C27" t="s">
         <v>36</v>
@@ -1907,7 +1970,7 @@
         <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C28" t="s">
         <v>63</v>
@@ -1921,7 +1984,7 @@
         <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C29" t="s">
         <v>63</v>
@@ -1932,7 +1995,7 @@
         <v>66</v>
       </c>
       <c r="B30" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C30" t="s">
         <v>63</v>
@@ -1943,7 +2006,7 @@
         <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C31" t="s">
         <v>63</v>
@@ -1954,7 +2017,7 @@
         <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C32" t="s">
         <v>63</v>
@@ -1968,10 +2031,13 @@
         <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C33" t="s">
         <v>63</v>
+      </c>
+      <c r="D33" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
@@ -1979,10 +2045,13 @@
         <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C34" t="s">
         <v>63</v>
+      </c>
+      <c r="D34" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -1990,10 +2059,13 @@
         <v>72</v>
       </c>
       <c r="B35" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C35" t="s">
         <v>63</v>
+      </c>
+      <c r="D35" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
@@ -2001,38 +2073,35 @@
         <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>156</v>
+        <v>228</v>
       </c>
       <c r="C36" t="s">
-        <v>157</v>
-      </c>
-      <c r="D36" t="s">
-        <v>74</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
-        <v>179</v>
+        <v>226</v>
       </c>
       <c r="C37" t="s">
         <v>33</v>
       </c>
       <c r="D37" t="s">
-        <v>76</v>
+        <v>227</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B38" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C38" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2045,111 +2114,125 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="43" style="1" customWidth="1"/>
+    <col min="3" max="3" width="39" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>23</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>25</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deposit the range-review decisions and apply them with a shared function
- Added a new Elev_max column, replacing the hard-coded Henicorhina exception in 04b
- flag_range_decisions() holds 04b's logic; Bird_pcs_dist.csv contents are unchanged
- Exported as DataS1/Spp_remove_change.csv; added definitions to Column_definitions_final.xlsx

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DataS1/Column_definitions_final.xlsx
+++ b/DataS1/Column_definitions_final.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/aaron_skinner2_ubc_ca/Documents/Academia/PhD/Analysis/Ssp-bird-data-wrangling/DataS1/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="164" documentId="11_2A7B806BDA388D21EAE73AD5D10BB879CF387425" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36ADA9C1-E8BC-CE41-8F1B-134B935CD0C9}"/>
   <bookViews>
-    <workbookView xWindow="1660" yWindow="660" windowWidth="25120" windowHeight="13180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4060" yWindow="1320" windowWidth="25120" windowHeight="13180" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bird_pcs_all" sheetId="1" r:id="rId1"/>
-    <sheet name="Event_covs" sheetId="6" r:id="rId2"/>
-    <sheet name="Site_covs" sheetId="3" r:id="rId3"/>
-    <sheet name="Functional_traits" sheetId="7" r:id="rId4"/>
-    <sheet name="Taxonomy" sheetId="5" r:id="rId5"/>
+    <sheet name="Bird_pcs_all" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Event_covs" sheetId="6" state="visible" r:id="rId2"/>
+    <sheet name="Site_covs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Functional_traits" sheetId="7" state="visible" r:id="rId4"/>
+    <sheet name="Taxonomy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Spp_remove_change" sheetId="8" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
   <si>
     <t>Field_name</t>
   </si>
@@ -748,18 +742,90 @@
   <si>
     <t>Generation length (Years)</t>
   </si>
+  <si>
+    <t xml:space="preserve">Field_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column_content_definition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species_ayerbe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species as reported in 'Bird_pcs_all' (Ayerbe-Quiñones 2018) to which the decision applies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species_changed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species the observations are reassigned to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filled only when Decision = 'Change'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Range-review decision applied to the observations of this species when building 'Bird_pcs_analysis'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove = observations excluded from 'Bird_pcs_analysis'; Change = observations reassigned to 'Species_changed'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Departments_affected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department(s) where the decision applies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comma-separated; blank = the decision applies in all departments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elev_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum elevation (m) at which the decision applies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The decision applies to point counts at or below this elevation; blank = all elevations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Who made the decision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nick = Nick Bayly; Aaron = Aaron Skinner; Gaica = Asociación GAICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale for the decision</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -782,10 +848,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1082,15 +1151,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="59.33203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="59.33203125" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1101,7 +1170,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1112,7 +1181,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -1120,7 +1189,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" t="s">
         <v>82</v>
       </c>
@@ -1128,7 +1197,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5" t="s">
         <v>83</v>
       </c>
@@ -1136,7 +1205,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -1144,7 +1213,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" t="s">
         <v>85</v>
       </c>
@@ -1155,7 +1224,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+    <row r="8" ht="80" customHeight="1">
       <c r="A8" t="s">
         <v>87</v>
       </c>
@@ -1167,7 +1236,7 @@
       </c>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" ht="96" x14ac:dyDescent="0.2">
+    <row r="9" ht="96" customHeight="1">
       <c r="A9" t="s">
         <v>88</v>
       </c>
@@ -1178,7 +1247,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="80" x14ac:dyDescent="0.2">
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" t="s">
         <v>90</v>
       </c>
@@ -1196,16 +1265,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="61.83203125" customWidth="1"/>
-    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="61.83203125" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1216,7 +1285,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1227,7 +1296,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -1235,7 +1304,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="144" x14ac:dyDescent="0.2">
+    <row r="4" ht="144" customHeight="1">
       <c r="A4" t="s">
         <v>92</v>
       </c>
@@ -1246,7 +1315,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+    <row r="5" ht="96" customHeight="1">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -1257,7 +1326,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -1265,7 +1334,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" t="s">
         <v>82</v>
       </c>
@@ -1273,7 +1342,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -1284,7 +1353,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9" t="s">
         <v>101</v>
       </c>
@@ -1292,7 +1361,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10" t="s">
         <v>102</v>
       </c>
@@ -1300,7 +1369,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11" t="s">
         <v>103</v>
       </c>
@@ -1308,7 +1377,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12" t="s">
         <v>104</v>
       </c>
@@ -1316,7 +1385,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" t="s">
         <v>83</v>
       </c>
@@ -1324,7 +1393,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14" t="s">
         <v>195</v>
       </c>
@@ -1335,7 +1404,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15">
       <c r="A15" t="s">
         <v>107</v>
       </c>
@@ -1343,7 +1412,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16">
       <c r="A16" t="s">
         <v>108</v>
       </c>
@@ -1351,7 +1420,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17">
       <c r="A17" t="s">
         <v>110</v>
       </c>
@@ -1359,7 +1428,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" t="s">
         <v>121</v>
       </c>
@@ -1370,7 +1439,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19">
       <c r="A19" t="s">
         <v>111</v>
       </c>
@@ -1378,7 +1447,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+    <row r="20" ht="96" customHeight="1">
       <c r="A20" t="s">
         <v>112</v>
       </c>
@@ -1389,7 +1458,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21" t="s">
         <v>114</v>
       </c>
@@ -1400,7 +1469,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="112" x14ac:dyDescent="0.2">
+    <row r="22" ht="112" customHeight="1">
       <c r="A22" t="s">
         <v>116</v>
       </c>
@@ -1411,7 +1480,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23">
       <c r="A23" t="s">
         <v>117</v>
       </c>
@@ -1422,7 +1491,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" ht="16" customHeight="1">
       <c r="A24" t="s">
         <v>119</v>
       </c>
@@ -1433,7 +1502,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25">
       <c r="A25" t="s">
         <v>122</v>
       </c>
@@ -1444,7 +1513,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26">
       <c r="A26" t="s">
         <v>124</v>
       </c>
@@ -1455,7 +1524,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27">
       <c r="A27" t="s">
         <v>126</v>
       </c>
@@ -1473,15 +1542,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="2" max="2" width="51.1640625" customWidth="1"/>
-    <col min="3" max="3" width="29.6640625" customWidth="1"/>
+    <col min="2" max="2" width="51.1640625" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1492,7 +1561,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -1500,7 +1569,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" t="s">
         <v>127</v>
       </c>
@@ -1511,7 +1580,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" t="s">
         <v>129</v>
       </c>
@@ -1522,7 +1591,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5" t="s">
         <v>131</v>
       </c>
@@ -1530,7 +1599,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" t="s">
         <v>133</v>
       </c>
@@ -1538,7 +1607,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" t="s">
         <v>135</v>
       </c>
@@ -1546,7 +1615,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" t="s">
         <v>146</v>
       </c>
@@ -1554,7 +1623,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9" t="s">
         <v>148</v>
       </c>
@@ -1562,7 +1631,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10" t="s">
         <v>150</v>
       </c>
@@ -1573,7 +1642,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11" t="s">
         <v>202</v>
       </c>
@@ -1581,7 +1650,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12" t="s">
         <v>137</v>
       </c>
@@ -1589,7 +1658,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" t="s">
         <v>139</v>
       </c>
@@ -1597,7 +1666,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14" t="s">
         <v>141</v>
       </c>
@@ -1605,7 +1674,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+    <row r="15" ht="80" customHeight="1">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -1616,7 +1685,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="192" x14ac:dyDescent="0.2">
+    <row r="16" ht="192" customHeight="1">
       <c r="A16" t="s">
         <v>144</v>
       </c>
@@ -1634,17 +1703,17 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" customWidth="1"/>
-    <col min="2" max="2" width="92.33203125" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" customWidth="1"/>
-    <col min="4" max="4" width="55.6640625" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="92.33203125" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="55.6640625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1658,7 +1727,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1669,7 +1738,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -1683,7 +1752,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1694,7 +1763,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1705,7 +1774,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1716,7 +1785,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1727,7 +1796,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -1738,7 +1807,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9" t="s">
         <v>41</v>
       </c>
@@ -1749,7 +1818,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -1760,7 +1829,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -1771,7 +1840,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -1782,7 +1851,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -1793,7 +1862,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -1804,7 +1873,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -1815,7 +1884,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -1829,7 +1898,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1843,7 +1912,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -1857,7 +1926,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1871,7 +1940,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20">
       <c r="A20" t="s">
         <v>52</v>
       </c>
@@ -1885,7 +1954,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21">
       <c r="A21" t="s">
         <v>53</v>
       </c>
@@ -1896,7 +1965,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -1907,7 +1976,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -1918,7 +1987,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1929,7 +1998,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25">
       <c r="A25" t="s">
         <v>57</v>
       </c>
@@ -1940,7 +2009,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26">
       <c r="A26" t="s">
         <v>58</v>
       </c>
@@ -1951,7 +2020,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27">
       <c r="A27" t="s">
         <v>60</v>
       </c>
@@ -1965,7 +2034,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28">
       <c r="A28" t="s">
         <v>62</v>
       </c>
@@ -1979,7 +2048,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29">
       <c r="A29" t="s">
         <v>65</v>
       </c>
@@ -1990,7 +2059,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30">
       <c r="A30" t="s">
         <v>66</v>
       </c>
@@ -2001,7 +2070,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31">
       <c r="A31" t="s">
         <v>67</v>
       </c>
@@ -2012,7 +2081,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32">
       <c r="A32" t="s">
         <v>68</v>
       </c>
@@ -2026,7 +2095,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33">
       <c r="A33" t="s">
         <v>70</v>
       </c>
@@ -2040,7 +2109,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34">
       <c r="A34" t="s">
         <v>71</v>
       </c>
@@ -2054,7 +2123,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35">
       <c r="A35" t="s">
         <v>72</v>
       </c>
@@ -2068,7 +2137,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -2079,7 +2148,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2093,7 +2162,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38">
       <c r="A38" t="s">
         <v>76</v>
       </c>
@@ -2111,16 +2180,16 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" customWidth="1"/>
-    <col min="2" max="2" width="43" style="1" customWidth="1"/>
-    <col min="3" max="3" width="39" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="43" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="39" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" ht="16" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2131,7 +2200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2139,7 +2208,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2147,7 +2216,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2155,7 +2224,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2163,7 +2232,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2171,7 +2240,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2182,7 +2251,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2190,7 +2259,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2201,7 +2270,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2212,7 +2281,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -2220,7 +2289,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -2228,7 +2297,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -2240,4 +2309,104 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="22.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="50.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="60.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>